<commit_message>
Regras adicionais e ajustes da pagina
</commit_message>
<xml_diff>
--- a/Lista de Magia Atualizado.xlsx
+++ b/Lista de Magia Atualizado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\DeskTop\Base Geral\Ideias e Criações\Criação\Meu RPG\Fantasia\Ficha de Personagem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8926629-D405-4164-B15A-53A6B57B8D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15414B19-1BD1-410C-9C53-BC7CD38A8C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{883E12BE-FA78-4EE6-9606-DD6916CDE4BB}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$P$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -5427,7 +5427,7 @@
         <v>2</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F45" s="5" t="s">
         <v>70</v>
@@ -5467,7 +5467,7 @@
         <v>6</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F46" s="5" t="s">
         <v>70</v>
@@ -5507,7 +5507,7 @@
         <v>8</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F47" s="5" t="s">
         <v>70</v>
@@ -15557,7 +15557,7 @@
         <v>10</v>
       </c>
       <c r="E296" s="5" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F296" s="5" t="s">
         <v>70</v>
@@ -23273,7 +23273,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q1" xr:uid="{C49BDCF5-293D-48D6-A770-F16CD77D0F30}"/>
+  <autoFilter ref="A1:P1" xr:uid="{C49BDCF5-293D-48D6-A770-F16CD77D0F30}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P294">
     <sortCondition ref="D2:D294"/>
   </sortState>

</xml_diff>